<commit_message>
2026/06/04 CRUD backup update
</commit_message>
<xml_diff>
--- a/back_end/data/warehouse_list.xlsx
+++ b/back_end/data/warehouse_list.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <x:bookViews>
-    <x:workbookView xWindow="0" yWindow="0" windowWidth="25340" windowHeight="9890" tabRatio="500"/>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="12350" windowHeight="6590" tabRatio="500"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="Sheet1" sheetId="1" r:id="rId4"/>
@@ -22,48 +22,369 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="105">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="106">
+  <x:si>
+    <x:t>http://211.239.173.91:8080/csdst/login.do</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://211.239.173.91:8080/bbtdst/login.do</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://211.239.173.90:8080/aurdst/login.do</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://211.239.173.91:8080/hlgdst/login.do</x:t>
+  </x:si>
+  <x:si>
+    <x:r>
+      <x:t>웹출고</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:rFont val="맑은 고딕"/>
+        <x:sz val="10"/>
+        <x:color rgb="ff000000"/>
+      </x:rPr>
+      <x:t>(통관분)_아이디</x:t>
+    </x:r>
+  </x:si>
+  <x:si>
+    <x:r>
+      <x:t>웹출고</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:rFont val="맑은 고딕"/>
+        <x:sz val="10"/>
+        <x:color rgb="ff000000"/>
+      </x:rPr>
+      <x:t>(통관분)_비밀번호</x:t>
+    </x:r>
+  </x:si>
+  <x:si>
+    <x:t>azy081011***</x:t>
+  </x:si>
+  <x:si>
+    <x:t>강동2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>대청</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고려</x:t>
+  </x:si>
+  <x:si>
+    <x:t>01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>아이디</x:t>
+  </x:si>
+  <x:si>
+    <x:t>계정</x:t>
+  </x:si>
+  <x:si>
+    <x:t>강동1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경인</x:t>
+  </x:si>
+  <x:si>
+    <x:t>창고</x:t>
+  </x:si>
+  <x:si>
+    <x:t>00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>삼진1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>주소</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SWC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>02</x:t>
+  </x:si>
+  <x:si>
+    <x:t>삼진2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>유상</x:t>
+  </x:si>
+  <x:si>
+    <x:t>대재</x:t>
+  </x:si>
+  <x:si>
+    <x:t>견우오아시스</x:t>
+  </x:si>
+  <x:si>
+    <x:t>비밀번호</x:t>
+  </x:si>
+  <x:si>
+    <x:t>삼일물류</x:t>
+  </x:si>
+  <x:si>
+    <x:t>프라자로지스</x:t>
+  </x:si>
+  <x:si>
+    <x:t>hcy1dst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>타사이트</x:t>
+  </x:si>
+  <x:si>
+    <x:t>06053</x:t>
+  </x:si>
+  <x:si>
+    <x:t>베이지박스투</x:t>
+  </x:si>
+  <x:si>
+    <x:t>이스트밸리</x:t>
+  </x:si>
+  <x:si>
+    <x:t>aurdst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>한라동탄</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AZ0810</x:t>
+  </x:si>
+  <x:si>
+    <x:t>효성냉장</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웹출고 계정</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0101</x:t>
+  </x:si>
+  <x:si>
+    <x:t>kidst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>scmdept</x:t>
+  </x:si>
+  <x:si>
+    <x:t>az08100</x:t>
+  </x:si>
+  <x:si>
+    <x:t>한라곤지암</x:t>
+  </x:si>
+  <x:si>
+    <x:t>estdst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>희창냉장</x:t>
+  </x:si>
+  <x:si>
+    <x:t>약식주소</x:t>
+  </x:si>
+  <x:si>
+    <x:t>plzdst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>jnsdst3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>kd2dst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>hdtdst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>오로라CS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>kd1dst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시에이치물류</x:t>
+  </x:si>
+  <x:si>
+    <x:t>nswdst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>hlgdst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>신우냉장</x:t>
+  </x:si>
+  <x:si>
+    <x:t>sjn2dst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AZ08100</x:t>
+  </x:si>
+  <x:si>
+    <x:t>sjn1dst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>chdst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>djedst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>scustcd</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dchdst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>sidst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>통관분 계정</x:t>
+  </x:si>
+  <x:si>
+    <x:t>swdst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>az0810</x:t>
+  </x:si>
+  <x:si>
+    <x:t>91:8080</x:t>
+  </x:si>
+  <x:si>
+    <x:t>bbtdst</x:t>
+  </x:si>
+  <x:si>
+    <x:r>
+      <x:t>ip</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:rFont val="맑은 고딕"/>
+        <x:sz val="10"/>
+        <x:color rgb="ff000000"/>
+      </x:rPr>
+      <x:t>포트</x:t>
+    </x:r>
+  </x:si>
+  <x:si>
+    <x:r>
+      <x:t>통관분</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:rFont val="맑은 고딕"/>
+        <x:sz val="10"/>
+        <x:color rgb="ff000000"/>
+      </x:rPr>
+      <x:t>_아이디</x:t>
+    </x:r>
+  </x:si>
+  <x:si>
+    <x:r>
+      <x:t>웹출고</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:rFont val="맑은 고딕"/>
+        <x:sz val="10"/>
+        <x:color rgb="ff000000"/>
+      </x:rPr>
+      <x:t>_아이디</x:t>
+    </x:r>
+  </x:si>
+  <x:si>
+    <x:t>http://211.239.173.91:8080/hdtdst/login.do</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://211.239.173.91:8080/jnsdst3/login.do</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://211.239.173.91:8080/plzdst/login.do</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://211.239.173.91:8080/dchdst/login.do</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://nwill.net/hcy1dst/login.do</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://211.239.173.91:8080/chdst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://coldwms.hyosung.com/login.do</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://211.239.173.90/kd1dst/login.do</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://nwill.net:8080/estdst/login.do</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://211.239.173.90/kidst/login.do</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://211.239.173.90/sjn1dst/login.do</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://nwill.net:8080/nswdst/login.do</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://211.239.173.90/sjn2dst/login.do</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://211.239.173.90/kd2dst/login.do</x:t>
+  </x:si>
   <x:si>
     <x:t>http://nwill.net:8080/swdst/login.do</x:t>
   </x:si>
   <x:si>
-    <x:t>http://211.239.173.90/sjn1dst/login.do</x:t>
-  </x:si>
-  <x:si>
-    <x:t>http://211.239.173.90/kd1dst/login.do</x:t>
-  </x:si>
-  <x:si>
     <x:t>http://nwill.net:8080/djedst/login.do</x:t>
   </x:si>
   <x:si>
     <x:t>http://nwill.net:8080/sidst/login.do</x:t>
   </x:si>
   <x:si>
-    <x:t>http://211.239.173.90/kd2dst/login.do</x:t>
-  </x:si>
-  <x:si>
-    <x:t>http://nwill.net:8080/nswdst/login.do</x:t>
-  </x:si>
-  <x:si>
-    <x:t>http://211.239.173.90/kidst/login.do</x:t>
-  </x:si>
-  <x:si>
-    <x:t>http://211.239.173.90/sjn2dst/login.do</x:t>
-  </x:si>
-  <x:si>
-    <x:t>http://nwill.net:8080/estdst/login.do</x:t>
-  </x:si>
-  <x:si>
-    <x:t>http://nwill.net/hcy1dst/login.do</x:t>
-  </x:si>
-  <x:si>
-    <x:t>http://211.239.173.91:8080/chdst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>http://coldwms.hyosung.com/login.do</x:t>
-  </x:si>
-  <x:si>
-    <x:t>http://211.239.173.91:8080/bbtdst/login.do</x:t>
+    <x:t>zenith15</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AZ0810000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>zenith150</x:t>
+  </x:si>
+  <x:si>
+    <x:t>azy0101*</x:t>
+  </x:si>
+  <x:si>
+    <x:t>에이스냉장(통합)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>azy0812*</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웹출고(통관분) 계정</x:t>
+  </x:si>
+  <x:si>
+    <x:t>akwkddbxhd</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AZ081000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>제니스(곤지암)</x:t>
+  </x:si>
+  <x:si>
+    <x:r>
+      <x:t>웹출고</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:rFont val="맑은 고딕"/>
+        <x:sz val="10"/>
+        <x:color rgb="ff000000"/>
+      </x:rPr>
+      <x:t>_비밀번호</x:t>
+    </x:r>
   </x:si>
   <x:si>
     <x:r>
@@ -79,341 +400,23 @@
     </x:r>
   </x:si>
   <x:si>
-    <x:r>
-      <x:t>웹출고</x:t>
-    </x:r>
-    <x:r>
-      <x:rPr>
-        <x:rFont val="맑은 고딕"/>
-        <x:sz val="10"/>
-        <x:color rgb="ff000000"/>
-      </x:rPr>
-      <x:t>_비밀번호</x:t>
-    </x:r>
-  </x:si>
-  <x:si>
-    <x:t>zenith150</x:t>
-  </x:si>
-  <x:si>
-    <x:t>zenith15</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AZ0810000</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AZ081000</x:t>
-  </x:si>
-  <x:si>
-    <x:t>akwkddbxhd</x:t>
-  </x:si>
-  <x:si>
-    <x:t>에이스냉장(통합)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웹출고(통관분) 계정</x:t>
-  </x:si>
-  <x:si>
-    <x:t>azy0812*</x:t>
-  </x:si>
-  <x:si>
-    <x:t>azy0101*</x:t>
-  </x:si>
-  <x:si>
-    <x:t>제니스(곤지암)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경인</x:t>
-  </x:si>
-  <x:si>
-    <x:t>유상</x:t>
-  </x:si>
-  <x:si>
-    <x:t>대청</x:t>
-  </x:si>
-  <x:si>
-    <x:t>고려</x:t>
-  </x:si>
-  <x:si>
-    <x:t>강동1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>창고</x:t>
-  </x:si>
-  <x:si>
-    <x:t>계정</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>00</x:t>
-  </x:si>
-  <x:si>
-    <x:t>01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>아이디</x:t>
-  </x:si>
-  <x:si>
-    <x:t>삼진2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>02</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SWC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>대재</x:t>
-  </x:si>
-  <x:si>
-    <x:t>삼진1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>강동2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>주소</x:t>
-  </x:si>
-  <x:si>
-    <x:r>
-      <x:t>웹출고</x:t>
-    </x:r>
-    <x:r>
-      <x:rPr>
-        <x:rFont val="맑은 고딕"/>
-        <x:sz val="10"/>
-        <x:color rgb="ff000000"/>
-      </x:rPr>
-      <x:t>(통관분)_아이디</x:t>
-    </x:r>
-  </x:si>
-  <x:si>
-    <x:r>
-      <x:t>웹출고</x:t>
-    </x:r>
-    <x:r>
-      <x:rPr>
-        <x:rFont val="맑은 고딕"/>
-        <x:sz val="10"/>
-        <x:color rgb="ff000000"/>
-      </x:rPr>
-      <x:t>(통관분)_비밀번호</x:t>
-    </x:r>
-  </x:si>
-  <x:si>
-    <x:t>azy081011***</x:t>
-  </x:si>
-  <x:si>
-    <x:t>삼일물류</x:t>
-  </x:si>
-  <x:si>
-    <x:t>타사이트</x:t>
-  </x:si>
-  <x:si>
-    <x:t>hcy1dst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>비밀번호</x:t>
-  </x:si>
-  <x:si>
-    <x:t>프라자로지스</x:t>
-  </x:si>
-  <x:si>
-    <x:t>aurdst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>이스트밸리</x:t>
-  </x:si>
-  <x:si>
-    <x:t>한라동탄</x:t>
-  </x:si>
-  <x:si>
-    <x:t>베이지박스투</x:t>
-  </x:si>
-  <x:si>
-    <x:t>견우오아시스</x:t>
-  </x:si>
-  <x:si>
-    <x:t>estdst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>오로라CS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>희창냉장</x:t>
-  </x:si>
-  <x:si>
-    <x:t>06053</x:t>
-  </x:si>
-  <x:si>
-    <x:t>jnsdst3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>시에이치물류</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웹출고 계정</x:t>
-  </x:si>
-  <x:si>
-    <x:t>신우냉장</x:t>
-  </x:si>
-  <x:si>
-    <x:t>az08100</x:t>
-  </x:si>
-  <x:si>
-    <x:t>효성냉장</x:t>
-  </x:si>
-  <x:si>
-    <x:t>kd1dst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>kd2dst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>plzdst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>hdtdst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>약식주소</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AZ0810</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0101</x:t>
-  </x:si>
-  <x:si>
-    <x:t>kidst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>scmdept</x:t>
-  </x:si>
-  <x:si>
-    <x:t>한라곤지암</x:t>
-  </x:si>
-  <x:si>
-    <x:t>nswdst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>swdst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>91:8080</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AZ08100</x:t>
-  </x:si>
-  <x:si>
-    <x:t>sidst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>sjn2dst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>sjn1dst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>scustcd</x:t>
-  </x:si>
-  <x:si>
-    <x:t>djedst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dchdst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>az0810</x:t>
-  </x:si>
-  <x:si>
-    <x:t>hlgdst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>chdst</x:t>
-  </x:si>
-  <x:si>
-    <x:t>통관분 계정</x:t>
-  </x:si>
-  <x:si>
-    <x:t>bbtdst</x:t>
-  </x:si>
-  <x:si>
-    <x:r>
-      <x:t>웹출고</x:t>
-    </x:r>
-    <x:r>
-      <x:rPr>
-        <x:rFont val="맑은 고딕"/>
-        <x:sz val="10"/>
-        <x:color rgb="ff000000"/>
-      </x:rPr>
-      <x:t>_아이디</x:t>
-    </x:r>
-  </x:si>
-  <x:si>
-    <x:r>
-      <x:t>ip</x:t>
-    </x:r>
-    <x:r>
-      <x:rPr>
-        <x:rFont val="맑은 고딕"/>
-        <x:sz val="10"/>
-        <x:color rgb="ff000000"/>
-      </x:rPr>
-      <x:t>포트</x:t>
-    </x:r>
-  </x:si>
-  <x:si>
-    <x:r>
-      <x:t>통관분</x:t>
-    </x:r>
-    <x:r>
-      <x:rPr>
-        <x:rFont val="맑은 고딕"/>
-        <x:sz val="10"/>
-        <x:color rgb="ff000000"/>
-      </x:rPr>
-      <x:t>_아이디</x:t>
-    </x:r>
-  </x:si>
-  <x:si>
-    <x:t>http://211.239.173.91:8080/plzdst/login.do</x:t>
-  </x:si>
-  <x:si>
-    <x:t>http://211.239.173.91:8080/dchdst/login.do</x:t>
-  </x:si>
-  <x:si>
-    <x:t>http://211.239.173.90:8080/aurdst/login.do</x:t>
-  </x:si>
-  <x:si>
-    <x:t>http://211.239.173.91:8080/jnsdst3/login.do</x:t>
-  </x:si>
-  <x:si>
-    <x:t>http://211.239.173.91:8080/hdtdst/login.do</x:t>
-  </x:si>
-  <x:si>
-    <x:t>http://211.239.173.91:8080/hlgdst/login.do</x:t>
+    <x:t>http://krcs.itfarm.co.kr/</x:t>
+  </x:si>
+  <x:si>
+    <x:t>http://gwfood.itfarm.co.kr/</x:t>
   </x:si>
   <x:si>
     <x:t>http://www.xn--hg4bn0j.kr/</x:t>
   </x:si>
   <x:si>
-    <x:t>http://gwfood.itfarm.co.kr/</x:t>
-  </x:si>
-  <x:si>
     <x:t>https://cs.acecs.co.kr/IL6/</x:t>
-  </x:si>
-  <x:si>
-    <x:t>http://krcs.itfarm.co.kr/</x:t>
   </x:si>
 </x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="14">
+  <x:fonts count="15">
     <x:font>
       <x:name val="Calibri"/>
       <x:sz val="11"/>
@@ -586,6 +589,31 @@
         </x:font>
       </mc:Fallback>
     </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:font hs:extension="1">
+          <x:name val="맑은 고딕"/>
+          <x:sz val="11"/>
+          <x:color rgb="ff0000ff"/>
+          <x:u/>
+          <hs:underlineShape val="solid"/>
+          <hs:underlineType val="1"/>
+          <hs:underlineColor rgb="ff0000ff"/>
+          <hs:size val="100"/>
+          <hs:ratio val="100"/>
+          <hs:spacing val="0"/>
+          <hs:offset val="0"/>
+        </x:font>
+      </mc:Choice>
+      <mc:Fallback>
+        <x:font>
+          <x:name val="맑은 고딕"/>
+          <x:sz val="11"/>
+          <x:color rgb="ff0000ff"/>
+          <x:u/>
+        </x:font>
+      </mc:Fallback>
+    </mc:AlternateContent>
   </x:fonts>
   <x:fills count="2">
     <x:fill>
@@ -633,7 +661,7 @@
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="15">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
@@ -671,6 +699,9 @@
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1377,22 +1408,22 @@
   <x:sheetData>
     <x:row r="1" spans="1:15" ht="15" customHeight="1">
       <x:c r="A1" s="3"/>
-      <x:c r="B1" s="13" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="C1" s="13"/>
-      <x:c r="D1" s="13" t="s">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="E1" s="13"/>
-      <x:c r="F1" s="13" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="G1" s="13"/>
-      <x:c r="H1" s="13" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="I1" s="13"/>
+      <x:c r="B1" s="14" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C1" s="14"/>
+      <x:c r="D1" s="14" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="E1" s="14"/>
+      <x:c r="F1" s="14" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="G1" s="14"/>
+      <x:c r="H1" s="14" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="I1" s="14"/>
       <x:c r="J1" s="3"/>
       <x:c r="K1" s="3"/>
       <x:c r="L1" s="4"/>
@@ -1402,60 +1433,60 @@
     </x:row>
     <x:row r="2" spans="1:15" ht="15" customHeight="1">
       <x:c r="A2" s="3" t="s">
-        <x:v>31</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B2" s="3" t="s">
-        <x:v>36</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C2" s="3" t="s">
-        <x:v>50</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D2" s="3" t="s">
-        <x:v>94</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="E2" s="3" t="s">
-        <x:v>14</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="F2" s="3" t="s">
-        <x:v>92</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="G2" s="3" t="s">
-        <x:v>15</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="H2" s="3" t="s">
-        <x:v>44</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I2" s="3" t="s">
-        <x:v>45</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J2" s="3" t="s">
-        <x:v>43</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="K2" s="3" t="s">
-        <x:v>48</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="L2" s="3" t="s">
-        <x:v>71</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="M2" s="3" t="s">
-        <x:v>93</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="N2" s="3" t="s">
-        <x:v>84</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="O2" s="3" t="s">
-        <x:v>75</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:15" ht="15" customHeight="1">
       <x:c r="A3" s="3" t="s">
-        <x:v>30</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B3" s="3" t="s">
-        <x:v>65</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="C3" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D3" s="3"/>
       <x:c r="E3" s="3"/>
@@ -1464,11 +1495,11 @@
       <x:c r="H3" s="3"/>
       <x:c r="I3" s="3"/>
       <x:c r="J3" s="5" t="s">
-        <x:v>2</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="K3" s="3"/>
       <x:c r="L3" s="3" t="s">
-        <x:v>67</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="M3" s="8">
         <x:v>90</x:v>
@@ -1477,35 +1508,35 @@
         <x:v>16466</x:v>
       </x:c>
       <x:c r="O3" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:15" ht="15" customHeight="1">
       <x:c r="A4" s="3" t="s">
-        <x:v>42</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D4" s="3"/>
       <x:c r="E4" s="3"/>
       <x:c r="F4" s="3" t="s">
-        <x:v>65</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G4" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="H4" s="3"/>
       <x:c r="I4" s="3"/>
       <x:c r="J4" s="10" t="s">
-        <x:v>5</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="K4" s="3"/>
       <x:c r="L4" s="3" t="s">
-        <x:v>68</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="M4" s="8">
         <x:v>90</x:v>
@@ -1514,18 +1545,18 @@
         <x:v>11802</x:v>
       </x:c>
       <x:c r="O4" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:15" ht="15" customHeight="1">
       <x:c r="A5" s="11" t="s">
-        <x:v>56</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D5" s="3"/>
       <x:c r="E5" s="3"/>
@@ -1534,7 +1565,7 @@
       <x:c r="H5" s="3"/>
       <x:c r="I5" s="3"/>
       <x:c r="J5" s="12" t="s">
-        <x:v>102</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="K5" s="6" t="b">
         <x:v>1</x:v>
@@ -1543,18 +1574,18 @@
       <x:c r="M5" s="8"/>
       <x:c r="N5" s="3"/>
       <x:c r="O5" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:15" ht="15" customHeight="1">
       <x:c r="A6" s="3" t="s">
-        <x:v>26</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B6" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C6" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D6" s="3"/>
       <x:c r="E6" s="3"/>
@@ -1563,11 +1594,11 @@
       <x:c r="H6" s="3"/>
       <x:c r="I6" s="3"/>
       <x:c r="J6" s="6" t="s">
-        <x:v>7</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="K6" s="3"/>
       <x:c r="L6" s="3" t="s">
-        <x:v>74</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="M6" s="8">
         <x:v>90</x:v>
@@ -1576,18 +1607,18 @@
         <x:v>18069</x:v>
       </x:c>
       <x:c r="O6" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:15" ht="15" customHeight="1">
       <x:c r="A7" s="11" t="s">
-        <x:v>29</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B7" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C7" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D7" s="3"/>
       <x:c r="E7" s="3"/>
@@ -1596,7 +1627,7 @@
       <x:c r="H7" s="3"/>
       <x:c r="I7" s="3"/>
       <x:c r="J7" s="12" t="s">
-        <x:v>104</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="K7" s="6" t="b">
         <x:v>1</x:v>
@@ -1605,100 +1636,100 @@
       <x:c r="M7" s="8"/>
       <x:c r="N7" s="3"/>
       <x:c r="O7" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:15" ht="15" customHeight="1">
       <x:c r="A8" s="3" t="s">
-        <x:v>40</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B8" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C8" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D8" s="3"/>
       <x:c r="E8" s="3"/>
       <x:c r="F8" s="3" t="s">
-        <x:v>65</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G8" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="H8" s="3" t="s">
-        <x:v>17</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="I8" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="J8" s="5" t="s">
-        <x:v>3</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="K8" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L8" s="3" t="s">
-        <x:v>85</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="M8" s="8"/>
       <x:c r="N8" s="3">
         <x:v>14686</x:v>
       </x:c>
       <x:c r="O8" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:15" ht="15" customHeight="1">
       <x:c r="A9" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B9" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C9" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D9" s="3"/>
       <x:c r="E9" s="3"/>
       <x:c r="F9" s="3" t="s">
-        <x:v>65</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G9" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="H9" s="3" t="s">
-        <x:v>17</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="I9" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="J9" s="6" t="s">
-        <x:v>96</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="K9" s="3"/>
       <x:c r="L9" s="3" t="s">
-        <x:v>86</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="M9" s="8" t="s">
-        <x:v>79</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="N9" s="3">
         <x:v>23012</x:v>
       </x:c>
       <x:c r="O9" s="3" t="s">
-        <x:v>35</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:15" ht="15" customHeight="1">
       <x:c r="A10" s="3" t="s">
-        <x:v>55</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C10" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D10" s="3"/>
       <x:c r="E10" s="3"/>
@@ -1707,11 +1738,11 @@
       <x:c r="H10" s="3"/>
       <x:c r="I10" s="3"/>
       <x:c r="J10" s="5" t="s">
-        <x:v>13</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K10" s="3"/>
       <x:c r="L10" s="3" t="s">
-        <x:v>91</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="M10" s="8">
         <x:v>1</x:v>
@@ -1720,37 +1751,37 @@
         <x:v>15319</x:v>
       </x:c>
       <x:c r="O10" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:15" ht="15" customHeight="1">
       <x:c r="A11" s="3" t="s">
-        <x:v>47</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C11" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D11" s="3"/>
       <x:c r="E11" s="3"/>
       <x:c r="F11" s="3" t="s">
-        <x:v>65</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G11" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="H11" s="3"/>
       <x:c r="I11" s="3"/>
       <x:c r="J11" s="5" t="s">
-        <x:v>4</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="K11" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L11" s="3" t="s">
-        <x:v>81</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="M11" s="8">
         <x:v>1</x:v>
@@ -1759,35 +1790,35 @@
         <x:v>16546</x:v>
       </x:c>
       <x:c r="O11" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:15" ht="15" customHeight="1">
       <x:c r="A12" s="3" t="s">
-        <x:v>41</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C12" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D12" s="3"/>
       <x:c r="E12" s="3"/>
       <x:c r="F12" s="3" t="s">
-        <x:v>65</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G12" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="H12" s="3"/>
       <x:c r="I12" s="3"/>
       <x:c r="J12" s="5" t="s">
-        <x:v>1</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="K12" s="3"/>
       <x:c r="L12" s="3" t="s">
-        <x:v>83</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="M12" s="8">
         <x:v>90</x:v>
@@ -1796,31 +1827,31 @@
         <x:v>12861</x:v>
       </x:c>
       <x:c r="O12" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:15" ht="15" customHeight="1">
       <x:c r="A13" s="3" t="s">
-        <x:v>37</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B13" s="3"/>
       <x:c r="C13" s="3"/>
       <x:c r="D13" s="3"/>
       <x:c r="E13" s="3"/>
       <x:c r="F13" s="3" t="s">
-        <x:v>65</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G13" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="H13" s="3"/>
       <x:c r="I13" s="3"/>
       <x:c r="J13" s="5" t="s">
-        <x:v>8</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="K13" s="3"/>
       <x:c r="L13" s="3" t="s">
-        <x:v>82</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="M13" s="8">
         <x:v>90</x:v>
@@ -1829,74 +1860,74 @@
         <x:v>12861</x:v>
       </x:c>
       <x:c r="O13" s="3" t="s">
-        <x:v>35</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:15" ht="15" customHeight="1">
       <x:c r="A14" s="3" t="s">
-        <x:v>62</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>65</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="E14" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F14" s="3"/>
       <x:c r="G14" s="3"/>
       <x:c r="H14" s="3"/>
       <x:c r="I14" s="3"/>
       <x:c r="J14" s="5" t="s">
-        <x:v>11</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="K14" s="6"/>
       <x:c r="L14" s="6" t="s">
-        <x:v>89</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="M14" s="9" t="s">
-        <x:v>79</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="N14" s="3">
         <x:v>16596</x:v>
       </x:c>
       <x:c r="O14" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:15" ht="15" customHeight="1">
       <x:c r="A15" s="3" t="s">
-        <x:v>64</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C15" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>16</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="E15" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F15" s="3"/>
       <x:c r="G15" s="3"/>
       <x:c r="H15" s="3"/>
       <x:c r="I15" s="3"/>
       <x:c r="J15" s="5" t="s">
-        <x:v>0</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="K15" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L15" s="6" t="s">
-        <x:v>78</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="M15" s="8">
         <x:v>1</x:v>
@@ -1905,31 +1936,31 @@
         <x:v>17040</x:v>
       </x:c>
       <x:c r="O15" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:15" ht="15" customHeight="1">
       <x:c r="A16" s="11" t="s">
-        <x:v>21</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
-        <x:v>72</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C16" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D16" s="3"/>
       <x:c r="E16" s="3"/>
       <x:c r="F16" s="3"/>
       <x:c r="G16" s="3"/>
       <x:c r="H16" s="3" t="s">
-        <x:v>80</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="I16" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="J16" s="12" t="s">
-        <x:v>103</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="K16" s="6" t="b">
         <x:v>1</x:v>
@@ -1938,35 +1969,35 @@
       <x:c r="M16" s="8"/>
       <x:c r="N16" s="3"/>
       <x:c r="O16" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:15" ht="15" customHeight="1">
       <x:c r="A17" s="3" t="s">
-        <x:v>58</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="B17" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C17" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D17" s="3"/>
       <x:c r="E17" s="3"/>
       <x:c r="F17" s="3" t="s">
-        <x:v>65</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G17" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="H17" s="3"/>
       <x:c r="I17" s="3"/>
       <x:c r="J17" s="5" t="s">
-        <x:v>97</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K17" s="6"/>
       <x:c r="L17" s="6" t="s">
-        <x:v>52</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="M17" s="9">
         <x:v>1</x:v>
@@ -1975,18 +2006,18 @@
         <x:v>18007</x:v>
       </x:c>
       <x:c r="O17" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:15" ht="15" customHeight="1">
       <x:c r="A18" s="11" t="s">
-        <x:v>27</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C18" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D18" s="3"/>
       <x:c r="E18" s="3"/>
@@ -1995,7 +2026,7 @@
       <x:c r="H18" s="3"/>
       <x:c r="I18" s="3"/>
       <x:c r="J18" s="12" t="s">
-        <x:v>101</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="K18" s="6" t="b">
         <x:v>1</x:v>
@@ -2004,18 +2035,18 @@
       <x:c r="M18" s="8"/>
       <x:c r="N18" s="6"/>
       <x:c r="O18" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:15" ht="15" customHeight="1">
       <x:c r="A19" s="3" t="s">
-        <x:v>53</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B19" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C19" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D19" s="3"/>
       <x:c r="E19" s="3"/>
@@ -2024,13 +2055,13 @@
       <x:c r="H19" s="3"/>
       <x:c r="I19" s="3"/>
       <x:c r="J19" s="5" t="s">
-        <x:v>9</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="K19" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L19" s="3" t="s">
-        <x:v>57</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="M19" s="8">
         <x:v>1</x:v>
@@ -2039,59 +2070,59 @@
         <x:v>17210</x:v>
       </x:c>
       <x:c r="O19" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:15" ht="15" customHeight="1">
       <x:c r="A20" s="3" t="s">
-        <x:v>25</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="B20" s="3" t="s">
-        <x:v>20</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="C20" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D20" s="3"/>
       <x:c r="E20" s="3"/>
       <x:c r="F20" s="3" t="s">
-        <x:v>65</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G20" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="H20" s="3" t="s">
-        <x:v>65</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="I20" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="J20" s="5" t="s">
-        <x:v>98</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="K20" s="3"/>
       <x:c r="L20" s="3" t="s">
-        <x:v>61</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="M20" s="8" t="s">
-        <x:v>79</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="N20" s="3" t="s">
-        <x:v>60</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="O20" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:15" ht="15" customHeight="1">
       <x:c r="A21" s="3" t="s">
-        <x:v>51</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B21" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C21" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D21" s="3"/>
       <x:c r="E21" s="3"/>
@@ -2100,130 +2131,130 @@
       <x:c r="H21" s="3"/>
       <x:c r="I21" s="3"/>
       <x:c r="J21" s="5" t="s">
-        <x:v>95</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="K21" s="3"/>
       <x:c r="L21" s="3" t="s">
-        <x:v>69</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="M21" s="8" t="s">
-        <x:v>79</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="N21" s="3">
         <x:v>21088</x:v>
       </x:c>
       <x:c r="O21" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:15" ht="15" customHeight="1">
       <x:c r="A22" s="3" t="s">
-        <x:v>76</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B22" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C22" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D22" s="3"/>
       <x:c r="E22" s="3"/>
       <x:c r="F22" s="3" t="s">
-        <x:v>65</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G22" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="H22" s="3" t="s">
-        <x:v>17</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="I22" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="J22" s="5" t="s">
-        <x:v>100</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K22" s="3"/>
       <x:c r="L22" s="3" t="s">
-        <x:v>88</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="M22" s="8" t="s">
-        <x:v>79</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="N22" s="3">
         <x:v>17186</x:v>
       </x:c>
       <x:c r="O22" s="3" t="s">
-        <x:v>35</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:15" ht="15" customHeight="1">
       <x:c r="A23" s="3" t="s">
-        <x:v>54</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B23" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C23" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D23" s="3"/>
       <x:c r="E23" s="3"/>
       <x:c r="F23" s="3" t="s">
-        <x:v>65</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G23" s="3" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="H23" s="3" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="I23" s="3" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="J23" s="5" t="s">
         <x:v>73</x:v>
-      </x:c>
-      <x:c r="H23" s="3" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I23" s="3" t="s">
-        <x:v>73</x:v>
-      </x:c>
-      <x:c r="J23" s="5" t="s">
-        <x:v>99</x:v>
       </x:c>
       <x:c r="K23" s="3"/>
       <x:c r="L23" s="3" t="s">
-        <x:v>70</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="M23" s="8" t="s">
-        <x:v>79</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="N23" s="3">
         <x:v>18402</x:v>
       </x:c>
       <x:c r="O23" s="3" t="s">
-        <x:v>38</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:15" ht="15" customHeight="1">
       <x:c r="A24" s="3" t="s">
-        <x:v>66</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
-        <x:v>19</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="C24" s="3" t="s">
-        <x:v>24</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="D24" s="3"/>
       <x:c r="E24" s="3"/>
       <x:c r="F24" s="3" t="s">
-        <x:v>19</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="G24" s="3" t="s">
-        <x:v>23</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="H24" s="3" t="s">
-        <x:v>18</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="I24" s="3" t="s">
-        <x:v>46</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="J24" s="5" t="s">
-        <x:v>12</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="K24" s="6" t="b">
         <x:v>1</x:v>
@@ -2236,18 +2267,18 @@
         <x:v>15755</x:v>
       </x:c>
       <x:c r="O24" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:15" ht="15" customHeight="1">
       <x:c r="A25" s="3" t="s">
-        <x:v>59</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C25" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D25" s="3"/>
       <x:c r="E25" s="3"/>
@@ -2256,13 +2287,13 @@
       <x:c r="H25" s="3"/>
       <x:c r="I25" s="3"/>
       <x:c r="J25" s="5" t="s">
-        <x:v>10</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="K25" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L25" s="3" t="s">
-        <x:v>49</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="M25" s="8">
         <x:v>1</x:v>
@@ -2271,74 +2302,70 @@
         <x:v>14674</x:v>
       </x:c>
       <x:c r="O25" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:15" ht="15" customHeight="1">
       <x:c r="A26" s="3" t="s">
-        <x:v>33</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C26" s="3" t="s">
-        <x:v>73</x:v>
-      </x:c>
-      <x:c r="D26" s="3" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="E26" s="3" t="s">
-        <x:v>73</x:v>
-      </x:c>
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="D26" s="3"/>
+      <x:c r="E26" s="3"/>
       <x:c r="F26" s="3"/>
       <x:c r="G26" s="3"/>
       <x:c r="H26" s="3"/>
       <x:c r="I26" s="3"/>
-      <x:c r="J26" s="5" t="s">
-        <x:v>99</x:v>
+      <x:c r="J26" s="13" t="s">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K26" s="3"/>
       <x:c r="L26" s="3" t="s">
-        <x:v>70</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="M26" s="8" t="s">
-        <x:v>79</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="N26" s="3">
-        <x:v>18402</x:v>
+        <x:v>17153</x:v>
       </x:c>
       <x:c r="O26" s="3" t="s">
-        <x:v>38</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:15" ht="15" customHeight="1">
       <x:c r="A27" s="3" t="s">
-        <x:v>39</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="B27" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C27" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D27" s="3" t="s">
-        <x:v>16</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="E27" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F27" s="3"/>
       <x:c r="G27" s="3"/>
       <x:c r="H27" s="3"/>
       <x:c r="I27" s="3"/>
       <x:c r="J27" s="5" t="s">
-        <x:v>6</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="K27" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L27" s="3" t="s">
-        <x:v>77</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="M27" s="8">
         <x:v>1</x:v>
@@ -2347,7 +2374,7 @@
         <x:v>17090</x:v>
       </x:c>
       <x:c r="O27" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2366,7 +2393,6 @@
     <x:hyperlink ref="J21:J21" r:id="rId5"/>
     <x:hyperlink ref="J22:J22" r:id="rId6"/>
     <x:hyperlink ref="J23:J23" r:id="rId7"/>
-    <x:hyperlink ref="J26:J26" r:id="rId7"/>
     <x:hyperlink ref="J27:J27" r:id="rId8"/>
     <x:hyperlink ref="J25:J25" r:id="rId9"/>
     <x:hyperlink ref="J19:J19" r:id="rId10"/>
@@ -2381,6 +2407,7 @@
     <x:hyperlink ref="J7:J7" r:id="rId19"/>
     <x:hyperlink ref="J16:J16" r:id="rId20"/>
     <x:hyperlink ref="J18:J18" r:id="rId21"/>
+    <x:hyperlink ref="J26:J26" r:id="rId22"/>
   </x:hyperlinks>
   <x:pageMargins left="0.69972223043441772" right="0.69972223043441772" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
   <x:pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" useFirstPageNumber="0" horizontalDpi="600" verticalDpi="600" copies="1"/>

</xml_diff>